<commit_message>
Remove local paths from workbooks and genericize a sample counterparty
Strip the saved workbook path and cached folder values, normalize author metadata, replace one sample counterparty name with a generic one and refresh the example screenshot.
</commit_message>
<xml_diff>
--- a/en/Statements.xlsx
+++ b/en/Statements.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ЭтаКнига" defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\valk\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280C9A11-C7B3-41E7-B9B6-5D45F0A0E1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25420" windowHeight="16300" activeTab="1" xr2:uid="{D5CA26CE-9EEC-4977-BB11-A06D7CD562E3}"/>
@@ -251,7 +246,7 @@
     <t>Bank C</t>
   </si>
   <si>
-    <t>ФГБУ "Росводоканал"</t>
+    <t>ФГБУ "Водоканал"</t>
   </si>
   <si>
     <t>Branch_D</t>
@@ -1594,7 +1589,7 @@
       </c>
       <c r="B2" t="str">
         <f ca="1">LEFT(CELL("filename",A1),FIND("[",CELL("filename",A1))-1)&amp;"Name Folder\"</f>
-        <v>C:\Users\valk\Downloads\Name Folder\</v>
+        <v>C:\Examples\Name Folder\</v>
       </c>
     </row>
   </sheetData>

</xml_diff>